<commit_message>
demo-ui-redesign story-002：基元描述数据层（GeneCatalog/OrganelleCatalog/EnemySpec 补 Description，CodexRegistry 统一图鉴查询接口）
CardSpec 已有 Desc/DetailDesc 不改；cell.CellEnemy 表新增 desc 字段并跑 Luban codegen。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#CellEnemy-敌人配置.xlsx
+++ b/Configs/GameConfig/Datas/cell/#CellEnemy-敌人配置.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,11 @@
           <t>isBoss</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -589,6 +594,11 @@
           <t>bool</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -674,6 +684,11 @@
       <c r="Q3" t="inlineStr">
         <is>
           <t>是否首领</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>机制说明（图鉴/tooltip，story-002）</t>
         </is>
       </c>
     </row>
@@ -731,6 +746,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>无害漂浮，纯资源，不主动攻击。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -790,6 +810,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>带刺膜不可直接吞噬，需先破防才能吃。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
@@ -845,6 +870,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>沿路径巡逻，靠近才会发现玩家。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -898,6 +928,11 @@
       <c r="Q7" t="inlineStr">
         <is>
           <t>False</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>直线追击玩家，基础威胁单位。</t>
         </is>
       </c>
     </row>
@@ -955,6 +990,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>成群出现，单体脆弱但数量多。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -1014,6 +1054,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>外壳坚硬且不可直接吞噬，需先破壳。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -1073,6 +1118,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>天生带电，电系连锁的理想引爆点。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -1132,6 +1182,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>自带污染状态，靠近易被感染。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -1187,6 +1242,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>冲撞式突进，攻击前有蓄力预警。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -1242,6 +1302,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>保持距离进行远程投射攻击。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -1297,6 +1362,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>固定不动，依靠原地范围输出。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -1352,6 +1422,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>低成本快速刷新，用于填充生态密度。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -1407,6 +1482,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>冲撞后近身吸取资源。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -1462,6 +1542,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>外观伪装，行为与低威胁单位相似。</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
@@ -1521,6 +1606,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>带腐蚀状态，接触会持续侵蚀。</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
@@ -1576,6 +1666,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>会主动追猎并吞噬其他弱小单位。</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -1635,6 +1730,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>血量与硬度极高，且不可直接吞噬。</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -1694,6 +1794,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>成群移动并带电，电系连锁的高密度目标。</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
@@ -1749,6 +1854,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>冲撞后附着在目标身上持续吸取。</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
@@ -1804,6 +1914,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>属性全面强化，进入后期的高威胁单位。</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
@@ -1863,6 +1978,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>精英：慢速但高血量，尝试直接追猎吞噬玩家。</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
@@ -1922,6 +2042,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>精英：绕轨环绕攻击，移速快难以摆脱。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
@@ -1981,6 +2106,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>精英：远程带电投射，配合电系连锁威胁大。</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
@@ -2040,6 +2170,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>精英：固守原地持续孵化威胁。</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
@@ -2099,6 +2234,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>精英：固守巢穴，坚硬难破防。</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
@@ -2158,6 +2298,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>精英：冲撞式突进，攻击凶猛。</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
@@ -2217,6 +2362,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>精英：远程虹吸，持续削弱玩家资源。</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
@@ -2276,6 +2426,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>精英：自带污染，接触持续侵蚀且血量高。</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
@@ -2335,6 +2490,11 @@
           <t>True</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>首领：三阶段血量切换行为，终局最高威胁目标。</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
@@ -2390,6 +2550,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>尸体/残块，卡牌生成的二次吞噬目标，不由导演采购。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>